<commit_message>
tabulky a grafy 27 done
</commit_message>
<xml_diff>
--- a/uloha27/uloha27.xlsx
+++ b/uloha27/uloha27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nemec\david\school\praktika\uloha27\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B002A34-01E7-440F-B1A2-37EB8F4D39BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A7D65D-3410-4DFD-9FDD-091DBC3825E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{635767DE-D7BD-46F5-96D6-3D4DDDEDB1B5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>U0 (V)</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>teor. eps0</t>
+  </si>
+  <si>
+    <t>materiál</t>
   </si>
 </sst>
 </file>
@@ -4093,6 +4096,9 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>31</v>
+      </c>
       <c r="B40" t="s">
         <v>3</v>
       </c>

</xml_diff>